<commit_message>
turbine level config change
</commit_message>
<xml_diff>
--- a/data/test_land_turbines.xlsx
+++ b/data/test_land_turbines.xlsx
@@ -450,10 +450,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>9.699999999999999</v>
+        <v>8.69</v>
       </c>
       <c r="D2" t="n">
-        <v>52.4</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="3">
@@ -468,10 +468,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>9.709999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D3" t="n">
-        <v>52.4</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="4">
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>9.719999999999999</v>
+        <v>8.709999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>52.4</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="5">
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9.729999999999999</v>
+        <v>8.719999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>52.4</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="6">
@@ -522,10 +522,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9.699999999999999</v>
+        <v>8.69</v>
       </c>
       <c r="D6" t="n">
-        <v>52.41</v>
+        <v>51.51</v>
       </c>
     </row>
     <row r="7">
@@ -540,10 +540,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9.709999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>52.41</v>
+        <v>51.51</v>
       </c>
     </row>
     <row r="8">
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9.719999999999999</v>
+        <v>8.709999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>52.41</v>
+        <v>51.51</v>
       </c>
     </row>
     <row r="9">
@@ -576,10 +576,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9.729999999999999</v>
+        <v>8.719999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>52.41</v>
+        <v>51.51</v>
       </c>
     </row>
     <row r="10">
@@ -594,10 +594,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9.699999999999999</v>
+        <v>8.69</v>
       </c>
       <c r="D10" t="n">
-        <v>52.42</v>
+        <v>51.52</v>
       </c>
     </row>
     <row r="11">
@@ -612,10 +612,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9.709999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>52.42</v>
+        <v>51.52</v>
       </c>
     </row>
     <row r="12">
@@ -630,10 +630,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9.719999999999999</v>
+        <v>8.709999999999999</v>
       </c>
       <c r="D12" t="n">
-        <v>52.42</v>
+        <v>51.52</v>
       </c>
     </row>
     <row r="13">
@@ -648,10 +648,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9.729999999999999</v>
+        <v>8.719999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>52.42</v>
+        <v>51.52</v>
       </c>
     </row>
     <row r="14">
@@ -666,10 +666,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9.699999999999999</v>
+        <v>8.69</v>
       </c>
       <c r="D14" t="n">
-        <v>52.43</v>
+        <v>51.53</v>
       </c>
     </row>
     <row r="15">
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9.709999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>52.43</v>
+        <v>51.53</v>
       </c>
     </row>
     <row r="16">
@@ -702,10 +702,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9.719999999999999</v>
+        <v>8.709999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>52.43</v>
+        <v>51.53</v>
       </c>
     </row>
     <row r="17">
@@ -720,10 +720,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>9.729999999999999</v>
+        <v>8.719999999999999</v>
       </c>
       <c r="D17" t="n">
-        <v>52.43</v>
+        <v>51.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>